<commit_message>
Add ZapGooIm 韻調聲 schemas and dicts without oversized NCL PDF.
The NCL-26128 PDF exceeds GitHub's 100MB limit, so it is gitignored and kept local only.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/101_BP+BPM聲韻調對照表.xlsx
+++ b/docs/101_BP+BPM聲韻調對照表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlanJui\work\rime-tlpa\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7499957-8E62-4701-A5E4-11F8945B47E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4BB552-A3D6-43D3-B622-CF0BE6096F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{D0BEA036-CBAE-4DB6-B3FC-C04A99F1A832}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{D0BEA036-CBAE-4DB6-B3FC-C04A99F1A832}"/>
   </bookViews>
   <sheets>
     <sheet name="聲母對照表" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="177">
   <si>
     <t>BP</t>
   </si>
@@ -760,12 +760,64 @@
     <t>白話字</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>阿中二式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>zi</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ci</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>si</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ʨ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>tsi</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>曾</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ʨʰ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>tshi</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>chhi</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>出</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ɕ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>時</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -828,29 +880,9 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="細明體"/>
-      <family val="3"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
       <name val="Microsoft JhengHei UI"/>
       <family val="2"/>
       <charset val="136"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Microsoft JhengHei"/>
-      <family val="2"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
@@ -889,6 +921,20 @@
       <color rgb="FFFF0000"/>
       <name val="Microsoft JhengHei UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="霞鶩文楷等寬 TC Medium"/>
+      <family val="3"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="霞鶩文楷等寬 TC Medium"/>
+      <family val="3"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="6">
@@ -970,7 +1016,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -983,31 +1029,16 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1025,35 +1056,44 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1417,687 +1457,754 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{780E5E98-C630-4915-9799-365193D6924F}">
-  <dimension ref="B1:J27"/>
-  <sheetFormatPr defaultRowHeight="29.25"/>
+  <dimension ref="B1:K27"/>
+  <sheetFormatPr defaultRowHeight="29.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="0.5" style="2" customWidth="1"/>
-    <col min="2" max="10" width="11.25" style="2" customWidth="1"/>
-    <col min="11" max="11" width="0.875" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="9" style="2"/>
+    <col min="2" max="11" width="11.25" style="2" customWidth="1"/>
+    <col min="12" max="12" width="0.875" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="3.75" customHeight="1"/>
-    <row r="2" spans="2:10">
-      <c r="B2" s="20" t="s">
+    <row r="1" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="I2" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="J2" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="K2" s="14" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="44.25">
-      <c r="B3" s="14" t="s">
+    <row r="3" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B3" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="5" t="s">
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="K3" s="15" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="2:10" ht="44.25">
-      <c r="B4" s="14" t="s">
+    <row r="4" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="I4" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="K4" s="15" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="44.25">
-      <c r="B5" s="14" t="s">
+    <row r="5" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B5" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="J5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J5" s="21" t="s">
+      <c r="K5" s="15" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="44.25">
-      <c r="B6" s="15" t="s">
+    <row r="6" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="I6" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="J6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="K6" s="16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="44.25">
-      <c r="B7" s="16" t="s">
+    <row r="7" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I7" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="J7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="K7" s="17" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="44.25">
-      <c r="B8" s="14" t="s">
+    <row r="8" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="I8" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="K8" s="15" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="2:10" ht="44.25">
-      <c r="B9" s="14" t="s">
+    <row r="9" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="I9" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="K9" s="15" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="2:10" ht="44.25">
-      <c r="B10" s="15" t="s">
+    <row r="10" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="I10" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="J10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J10" s="22" t="s">
+      <c r="K10" s="16" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="11" spans="2:10" ht="44.25">
-      <c r="B11" s="16" t="s">
+    <row r="11" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="J11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="23" t="s">
+      <c r="K11" s="17" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="12" spans="2:10" ht="44.25">
-      <c r="B12" s="14" t="s">
+    <row r="12" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="J12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="K12" s="15" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="2:10" ht="44.25">
-      <c r="B13" s="14" t="s">
+    <row r="13" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="J13" s="21" t="s">
+      <c r="K13" s="15" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="44.25">
-      <c r="B14" s="15" t="s">
+    <row r="14" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B14" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="I14" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="J14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="J14" s="22" t="s">
+      <c r="K14" s="16" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="2:10" ht="44.25">
-      <c r="B15" s="16" t="s">
+    <row r="15" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B15" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="J15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="J15" s="23" t="s">
+      <c r="K15" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="2:10" ht="44.25">
-      <c r="B16" s="14" t="s">
+    <row r="16" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="14" t="s">
+      <c r="G16" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I16" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="J16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="J16" s="21" t="s">
+      <c r="K16" s="15" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="44.25">
-      <c r="B17" s="17" t="s">
+    <row r="17" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B17" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="12" t="s">
         <v>114</v>
       </c>
       <c r="H17" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="I17" s="13" t="s">
+      <c r="J17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J17" s="24" t="s">
+      <c r="K17" s="18" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="44.25">
-      <c r="B18" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="18" t="s">
+    <row r="18" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B18" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B19" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I19" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B21" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="G21" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="H21" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="I21" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="I18" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="J18" s="21" t="s">
+      <c r="J21" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="K21" s="16" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="44.25">
-      <c r="B19" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="44.25">
-      <c r="B20" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" s="18" t="s">
+    <row r="22" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B22" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="G22" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H22" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="I22" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="I20" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="J20" s="21" t="s">
+      <c r="J22" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="K22" s="16" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="44.25">
-      <c r="B21" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="I21" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" s="24" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" ht="44.25">
-      <c r="B22" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G22" s="18" t="s">
+    <row r="23" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B23" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="G23" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H23" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="I23" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="I22" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="J22" s="21" t="s">
+      <c r="J23" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="K23" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="2:10" ht="44.25">
-      <c r="B23" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="H23" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J23" s="22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" ht="44.25">
-      <c r="B24" s="15" t="s">
+    <row r="24" spans="2:11" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="B24" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="H24" s="11" t="s">
+      <c r="H24" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="I24" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="J24" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="J24" s="22" t="s">
+      <c r="K24" s="16" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="6.75" customHeight="1"/>
-    <row r="26" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B26" s="26" t="s">
+    <row r="25" spans="2:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="2:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="E26" s="25" t="s">
+      <c r="E26" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="19" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="9.75" customHeight="1"/>
+    <row r="27" spans="2:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2107,14 +2214,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F3C4FAB-5E39-4D8D-A6FB-D3D342E6E117}">
   <dimension ref="B2:V29"/>
-  <sheetFormatPr defaultRowHeight="29.25"/>
+  <sheetFormatPr defaultRowHeight="29.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.875" style="2" customWidth="1"/>
     <col min="2" max="2" width="18.25" style="2" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:22">
+    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2179,7 +2286,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:22">
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
@@ -2244,7 +2351,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:22">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>30</v>
       </c>
@@ -2309,7 +2416,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="2:22">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>62</v>
       </c>
@@ -2374,7 +2481,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="2:22">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>50</v>
       </c>
@@ -2439,7 +2546,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="2:22">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>0</v>
       </c>
@@ -2456,7 +2563,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="2:22">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
@@ -2473,7 +2580,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:22">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>2</v>
       </c>
@@ -2490,7 +2597,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:22">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
@@ -2507,7 +2614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:22">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
@@ -2524,7 +2631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:22">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>5</v>
       </c>
@@ -2541,7 +2648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="2:22">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>6</v>
       </c>
@@ -2558,7 +2665,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="2:22">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>7</v>
       </c>
@@ -2575,7 +2682,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:6">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
@@ -2592,7 +2699,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:6">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
@@ -2609,7 +2716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="2:6">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>10</v>
       </c>
@@ -2626,7 +2733,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="2:6">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>11</v>
       </c>
@@ -2643,7 +2750,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="2:6">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>12</v>
       </c>
@@ -2660,7 +2767,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="2:6">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>13</v>
       </c>
@@ -2677,7 +2784,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="2:6">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
         <v>14</v>
       </c>
@@ -2694,7 +2801,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="2:6">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
         <v>15</v>
       </c>
@@ -2711,7 +2818,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="2:6">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>16</v>
       </c>
@@ -2728,7 +2835,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="2:6">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2745,7 +2852,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="2:6">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
         <v>18</v>
       </c>
@@ -2762,7 +2869,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="2:6">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
         <v>19</v>
       </c>
@@ -2779,7 +2886,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="2:6">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="2" t="s">
         <v>20</v>
       </c>

</xml_diff>